<commit_message>
Fix fig 3 in ICS rmd
</commit_message>
<xml_diff>
--- a/AutoReadUSBRData/ReservoirElevationDefinitions.xlsx
+++ b/AutoReadUSBRData/ReservoirElevationDefinitions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Rosenberg\Work\USU\Research\ColoradoRiver\RCode\ColoradoRiverCollaborate\AutoReadUSBRData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F709FE7D-2B49-410C-91FC-622D0EFFE391}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DFC55C8-2F6D-4B29-9BF8-1082124F75A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{8459C475-5003-475B-AAB9-94E9EA45958F}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{8459C475-5003-475B-AAB9-94E9EA45958F}"/>
   </bookViews>
   <sheets>
     <sheet name="ReadMe" sheetId="2" r:id="rId1"/>
@@ -42,9 +42,6 @@
     <t>Protect (2026 DEIS)</t>
   </si>
   <si>
-    <t>SNWA Intake #2</t>
-  </si>
-  <si>
     <t>Protect (2019 DCP)</t>
   </si>
   <si>
@@ -100,6 +97,9 @@
   </si>
   <si>
     <t>Elevation (feet)</t>
+  </si>
+  <si>
+    <t>Protect (2022 SEIS)</t>
   </si>
 </sst>
 </file>
@@ -969,31 +969,31 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -1005,16 +1005,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8FD67FD-F240-49E2-BF91-7D417E153654}">
   <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="16.90625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D1" t="s">
         <v>1</v>
@@ -1058,7 +1061,7 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="C5">
         <v>1000</v>
@@ -1069,7 +1072,7 @@
         <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C6">
         <v>1020</v>
@@ -1080,7 +1083,7 @@
         <v>2</v>
       </c>
       <c r="B7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C7">
         <v>1025</v>
@@ -1091,7 +1094,7 @@
         <v>2</v>
       </c>
       <c r="B8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C8">
         <v>1050</v>
@@ -1102,7 +1105,7 @@
         <v>2</v>
       </c>
       <c r="B9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C9">
         <v>1090</v>
@@ -1113,7 +1116,7 @@
         <v>2</v>
       </c>
       <c r="B10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C10">
         <v>1135</v>
@@ -1124,7 +1127,7 @@
         <v>2</v>
       </c>
       <c r="B11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C11">
         <v>1218</v>
@@ -1145,10 +1148,10 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D1" t="s">
         <v>1</v>
@@ -1156,10 +1159,10 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
         <v>13</v>
-      </c>
-      <c r="B2" t="s">
-        <v>14</v>
       </c>
       <c r="C2">
         <v>3370</v>
@@ -1167,7 +1170,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
         <v>4</v>
@@ -1178,7 +1181,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
         <v>5</v>
@@ -1189,10 +1192,10 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C5">
         <v>3525</v>
@@ -1200,10 +1203,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C6">
         <v>3575</v>
@@ -1211,10 +1214,10 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C7">
         <v>3600</v>
@@ -1222,10 +1225,10 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C8">
         <v>3700</v>

</xml_diff>

<commit_message>
Filter key Powell Elevations on Figure 4 Powell x Mead plot
</commit_message>
<xml_diff>
--- a/AutoReadUSBRData/ReservoirElevationDefinitions.xlsx
+++ b/AutoReadUSBRData/ReservoirElevationDefinitions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Rosenberg\Work\USU\Research\ColoradoRiver\RCode\ColoradoRiverCollaborate\AutoReadUSBRData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DFC55C8-2F6D-4B29-9BF8-1082124F75A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{778446EA-3379-45EB-863A-14C8A8F88A58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{8459C475-5003-475B-AAB9-94E9EA45958F}"/>
+    <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{8459C475-5003-475B-AAB9-94E9EA45958F}"/>
   </bookViews>
   <sheets>
     <sheet name="ReadMe" sheetId="2" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="29">
   <si>
     <t>Reservoir</t>
   </si>
@@ -100,6 +100,15 @@
   </si>
   <si>
     <t>Protect (2022 SEIS)</t>
+  </si>
+  <si>
+    <t>Turbines</t>
+  </si>
+  <si>
+    <t>Catastrophic - Turbine Vortices</t>
+  </si>
+  <si>
+    <t>Minimum Drawdown</t>
   </si>
 </sst>
 </file>
@@ -1140,8 +1149,12 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E38887C4-AA44-419C-B405-A9906CF058A2}">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="10.08984375" customWidth="1"/>
+    <col min="2" max="2" width="16.36328125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
@@ -1173,7 +1186,7 @@
         <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="C3">
         <v>3490</v>
@@ -1195,10 +1208,10 @@
         <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="C5">
-        <v>3525</v>
+        <v>3514</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
@@ -1206,10 +1219,10 @@
         <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="C6">
-        <v>3575</v>
+        <v>3525</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
@@ -1217,10 +1230,10 @@
         <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="C7">
-        <v>3600</v>
+        <v>3550</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
@@ -1228,9 +1241,31 @@
         <v>12</v>
       </c>
       <c r="B8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8">
+        <v>3575</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9">
+        <v>3600</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" t="s">
         <v>14</v>
       </c>
-      <c r="C8">
+      <c r="C10">
         <v>3700</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fixed plot on .R
</commit_message>
<xml_diff>
--- a/AutoReadUSBRData/ReservoirElevationDefinitions.xlsx
+++ b/AutoReadUSBRData/ReservoirElevationDefinitions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Rosenberg\Work\USU\Research\ColoradoRiver\RCode\ColoradoRiverCollaborate\AutoReadUSBRData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8D719C3-2BC5-42D1-8879-024D72A9E944}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D37831BC-877F-48EF-A10D-FF2924633264}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{8459C475-5003-475B-AAB9-94E9EA45958F}"/>
   </bookViews>
@@ -108,7 +108,7 @@
     <t>No Turbines (Vortices)</t>
   </si>
   <si>
-    <t>Potential Buffer</t>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Adjustments to text labels for Buffer and Catastrophic elevations
</commit_message>
<xml_diff>
--- a/AutoReadUSBRData/ReservoirElevationDefinitions.xlsx
+++ b/AutoReadUSBRData/ReservoirElevationDefinitions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Rosenberg\Work\USU\Research\ColoradoRiver\RCode\ColoradoRiverCollaborate\AutoReadUSBRData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1ED93D4-7D91-4728-BD26-15559E406195}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A4741D9-F0FF-4F19-AC5F-4E935F837BB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{8459C475-5003-475B-AAB9-94E9EA45958F}"/>
   </bookViews>
@@ -102,13 +102,13 @@
     <t>Protect (2022 SEIS)</t>
   </si>
   <si>
-    <t>Turbines</t>
-  </si>
-  <si>
-    <t>No Penstocks (Vortices)</t>
-  </si>
-  <si>
     <t>2x Buffer Volume</t>
+  </si>
+  <si>
+    <t>Top of Penstocks</t>
+  </si>
+  <si>
+    <t>No Hydropower (Vortices)</t>
   </si>
 </sst>
 </file>
@@ -1186,7 +1186,7 @@
         <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C3">
         <v>3490</v>
@@ -1208,7 +1208,7 @@
         <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C5">
         <v>3514</v>
@@ -1230,7 +1230,7 @@
         <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C7">
         <v>3535</v>

</xml_diff>